<commit_message>
Deploy preview for PR 101 🛫
</commit_message>
<xml_diff>
--- a/pr-preview/pr-101/assets/coremeta4cat_vocabulary.xlsx
+++ b/pr-preview/pr-101/assets/coremeta4cat_vocabulary.xlsx
@@ -1711,7 +1711,7 @@
       <c r="H10" s="13" t="inlineStr"/>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>CHEBI:52717</t>
+          <t>VOC4CAT:0007794</t>
         </is>
       </c>
       <c r="J10" s="13" t="inlineStr">
@@ -1906,7 +1906,7 @@
       <c r="H15" s="13" t="inlineStr"/>
       <c r="I15" s="13" t="inlineStr">
         <is>
-          <t>OBI:0000272</t>
+          <t>VOC4CAT:0007016</t>
         </is>
       </c>
       <c r="J15" s="13" t="inlineStr">
@@ -2076,7 +2076,7 @@
       <c r="H19" s="13" t="inlineStr"/>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J19" s="13" t="inlineStr">
@@ -2168,7 +2168,7 @@
       <c r="H21" s="12" t="inlineStr"/>
       <c r="I21" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J21" s="12" t="inlineStr">
@@ -2208,7 +2208,7 @@
       <c r="H22" s="12" t="inlineStr"/>
       <c r="I22" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J22" s="12" t="inlineStr">
@@ -2248,7 +2248,7 @@
       <c r="H23" s="12" t="inlineStr"/>
       <c r="I23" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J23" s="12" t="inlineStr">
@@ -2284,7 +2284,7 @@
       <c r="H24" s="13" t="inlineStr"/>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J24" s="13" t="inlineStr">
@@ -2332,7 +2332,7 @@
       <c r="H25" s="12" t="inlineStr"/>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J25" s="12" t="inlineStr">
@@ -2592,7 +2592,7 @@
       <c r="H32" s="12" t="inlineStr"/>
       <c r="I32" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000060</t>
         </is>
       </c>
       <c r="J32" s="12" t="inlineStr">
@@ -2628,7 +2628,7 @@
       <c r="H33" s="13" t="inlineStr"/>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J33" s="13" t="inlineStr">
@@ -2833,7 +2833,7 @@
       <c r="H38" s="13" t="inlineStr"/>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J38" s="13" t="inlineStr">
@@ -2873,7 +2873,7 @@
       <c r="H39" s="12" t="inlineStr"/>
       <c r="I39" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000056</t>
         </is>
       </c>
       <c r="J39" s="12" t="inlineStr">
@@ -3210,7 +3210,7 @@
       <c r="H48" s="13" t="inlineStr"/>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr">
@@ -3462,7 +3462,7 @@
       <c r="H54" s="12" t="inlineStr"/>
       <c r="I54" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008204</t>
         </is>
       </c>
       <c r="J54" s="12" t="inlineStr">
@@ -3498,7 +3498,7 @@
       <c r="H55" s="13" t="inlineStr"/>
       <c r="I55" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J55" s="13" t="inlineStr">
@@ -3542,7 +3542,7 @@
       <c r="H56" s="12" t="inlineStr"/>
       <c r="I56" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J56" s="12" t="inlineStr">
@@ -3582,7 +3582,7 @@
       <c r="H57" s="12" t="inlineStr"/>
       <c r="I57" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J57" s="12" t="inlineStr">
@@ -3622,7 +3622,7 @@
       <c r="H58" s="12" t="inlineStr"/>
       <c r="I58" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J58" s="12" t="inlineStr">
@@ -3670,7 +3670,7 @@
       <c r="H59" s="12" t="inlineStr"/>
       <c r="I59" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J59" s="12" t="inlineStr">
@@ -3751,7 +3751,7 @@
       <c r="H61" s="12" t="inlineStr"/>
       <c r="I61" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000060</t>
         </is>
       </c>
       <c r="J61" s="12" t="inlineStr">
@@ -3923,7 +3923,7 @@
       <c r="H65" s="12" t="inlineStr"/>
       <c r="I65" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000056</t>
         </is>
       </c>
       <c r="J65" s="12" t="inlineStr">
@@ -4044,7 +4044,7 @@
       <c r="H68" s="12" t="inlineStr"/>
       <c r="I68" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008204</t>
         </is>
       </c>
       <c r="J68" s="12" t="inlineStr">
@@ -4176,7 +4176,7 @@
       <c r="H71" s="12" t="inlineStr"/>
       <c r="I71" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J71" s="12" t="inlineStr">
@@ -4216,7 +4216,7 @@
       <c r="H72" s="12" t="inlineStr"/>
       <c r="I72" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J72" s="12" t="inlineStr">
@@ -4256,7 +4256,7 @@
       <c r="H73" s="12" t="inlineStr"/>
       <c r="I73" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J73" s="12" t="inlineStr">
@@ -4304,7 +4304,7 @@
       <c r="H74" s="12" t="inlineStr"/>
       <c r="I74" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J74" s="12" t="inlineStr">
@@ -4433,7 +4433,7 @@
       <c r="H77" s="12" t="inlineStr"/>
       <c r="I77" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:stirrer_type</t>
+          <t>VOC4CAT:0008113</t>
         </is>
       </c>
       <c r="J77" s="12" t="inlineStr">
@@ -4517,7 +4517,7 @@
       <c r="H79" s="13" t="inlineStr"/>
       <c r="I79" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J79" s="13" t="inlineStr">
@@ -4649,7 +4649,7 @@
       <c r="H82" s="13" t="inlineStr"/>
       <c r="I82" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J82" s="13" t="inlineStr">
@@ -4782,7 +4782,7 @@
       <c r="H85" s="12" t="inlineStr"/>
       <c r="I85" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J85" s="12" t="inlineStr">
@@ -5068,7 +5068,7 @@
       <c r="H92" s="13" t="inlineStr"/>
       <c r="I92" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J92" s="13" t="inlineStr">
@@ -5308,7 +5308,7 @@
       <c r="H97" s="12" t="inlineStr"/>
       <c r="I97" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J97" s="12" t="inlineStr">
@@ -5761,7 +5761,7 @@
       <c r="H107" s="12" t="inlineStr"/>
       <c r="I107" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J107" s="12" t="inlineStr">
@@ -6248,7 +6248,7 @@
       <c r="H118" s="13" t="inlineStr"/>
       <c r="I118" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J118" s="13" t="inlineStr">
@@ -6692,7 +6692,7 @@
       <c r="H129" s="12" t="inlineStr"/>
       <c r="I129" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008204</t>
         </is>
       </c>
       <c r="J129" s="12" t="inlineStr">
@@ -6736,7 +6736,7 @@
       <c r="H130" s="12" t="inlineStr"/>
       <c r="I130" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J130" s="12" t="inlineStr">
@@ -6776,7 +6776,7 @@
       <c r="H131" s="12" t="inlineStr"/>
       <c r="I131" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J131" s="12" t="inlineStr">
@@ -6816,7 +6816,7 @@
       <c r="H132" s="12" t="inlineStr"/>
       <c r="I132" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J132" s="12" t="inlineStr">
@@ -6864,7 +6864,7 @@
       <c r="H133" s="12" t="inlineStr"/>
       <c r="I133" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J133" s="12" t="inlineStr">
@@ -6945,7 +6945,7 @@
       <c r="H135" s="12" t="inlineStr"/>
       <c r="I135" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000060</t>
         </is>
       </c>
       <c r="J135" s="12" t="inlineStr">
@@ -7117,7 +7117,7 @@
       <c r="H139" s="12" t="inlineStr"/>
       <c r="I139" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000056</t>
         </is>
       </c>
       <c r="J139" s="12" t="inlineStr">
@@ -7442,7 +7442,7 @@
       <c r="H146" s="12" t="inlineStr"/>
       <c r="I146" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J146" s="12" t="inlineStr">
@@ -7651,7 +7651,7 @@
       <c r="H151" s="12" t="inlineStr"/>
       <c r="I151" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J151" s="12" t="inlineStr">
@@ -7691,7 +7691,7 @@
       <c r="H152" s="12" t="inlineStr"/>
       <c r="I152" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J152" s="12" t="inlineStr">
@@ -7731,7 +7731,7 @@
       <c r="H153" s="12" t="inlineStr"/>
       <c r="I153" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J153" s="12" t="inlineStr">
@@ -7779,7 +7779,7 @@
       <c r="H154" s="12" t="inlineStr"/>
       <c r="I154" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J154" s="12" t="inlineStr">
@@ -7860,7 +7860,7 @@
       <c r="H156" s="12" t="inlineStr"/>
       <c r="I156" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000060</t>
         </is>
       </c>
       <c r="J156" s="12" t="inlineStr">
@@ -8032,7 +8032,7 @@
       <c r="H160" s="12" t="inlineStr"/>
       <c r="I160" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000056</t>
         </is>
       </c>
       <c r="J160" s="12" t="inlineStr">
@@ -9058,7 +9058,7 @@
       <c r="H183" s="12" t="inlineStr"/>
       <c r="I183" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J183" s="12" t="inlineStr">
@@ -9335,7 +9335,7 @@
       <c r="H189" s="12" t="inlineStr"/>
       <c r="I189" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J189" s="12" t="inlineStr">
@@ -9536,7 +9536,7 @@
       <c r="H194" s="13" t="inlineStr"/>
       <c r="I194" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J194" s="13" t="inlineStr">
@@ -9828,7 +9828,7 @@
       <c r="H201" s="12" t="inlineStr"/>
       <c r="I201" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:precipitation_agent</t>
+          <t>VOC4CAT:0008203</t>
         </is>
       </c>
       <c r="J201" s="12" t="inlineStr">
@@ -10060,7 +10060,7 @@
       <c r="H206" s="12" t="inlineStr"/>
       <c r="I206" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J206" s="12" t="inlineStr">
@@ -10104,7 +10104,7 @@
       <c r="H207" s="12" t="inlineStr"/>
       <c r="I207" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:drying_device</t>
+          <t>VOC4CAT:0008122</t>
         </is>
       </c>
       <c r="J207" s="12" t="inlineStr">
@@ -10144,7 +10144,7 @@
       <c r="H208" s="12" t="inlineStr"/>
       <c r="I208" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008207</t>
         </is>
       </c>
       <c r="J208" s="12" t="inlineStr">
@@ -10184,7 +10184,7 @@
       <c r="H209" s="12" t="inlineStr"/>
       <c r="I209" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008206</t>
         </is>
       </c>
       <c r="J209" s="12" t="inlineStr">
@@ -10232,7 +10232,7 @@
       <c r="H210" s="12" t="inlineStr"/>
       <c r="I210" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0008208</t>
         </is>
       </c>
       <c r="J210" s="12" t="inlineStr">
@@ -10350,7 +10350,7 @@
       <c r="H213" s="12" t="inlineStr"/>
       <c r="I213" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000060</t>
         </is>
       </c>
       <c r="J213" s="12" t="inlineStr">
@@ -10522,7 +10522,7 @@
       <c r="H217" s="12" t="inlineStr"/>
       <c r="I217" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0000056</t>
         </is>
       </c>
       <c r="J217" s="12" t="inlineStr">
@@ -11270,7 +11270,7 @@
       <c r="H18" s="12" t="inlineStr"/>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J18" s="12" t="inlineStr">
@@ -11536,7 +11536,7 @@
       <c r="H25" s="13" t="inlineStr"/>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J25" s="13" t="inlineStr">
@@ -12490,7 +12490,7 @@
       <c r="H48" s="13" t="inlineStr"/>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr">
@@ -12882,7 +12882,7 @@
       <c r="H57" s="12" t="inlineStr"/>
       <c r="I57" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J57" s="12" t="inlineStr">
@@ -13215,7 +13215,7 @@
       <c r="H65" s="13" t="inlineStr"/>
       <c r="I65" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J65" s="13" t="inlineStr">
@@ -13681,7 +13681,7 @@
       <c r="H76" s="12" t="inlineStr"/>
       <c r="I76" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J76" s="12" t="inlineStr">
@@ -13814,7 +13814,7 @@
       <c r="H79" s="12" t="inlineStr"/>
       <c r="I79" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J79" s="12" t="inlineStr">
@@ -14551,7 +14551,7 @@
       <c r="H97" s="13" t="inlineStr"/>
       <c r="I97" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J97" s="13" t="inlineStr">
@@ -14643,7 +14643,7 @@
       <c r="H99" s="12" t="inlineStr"/>
       <c r="I99" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J99" s="12" t="inlineStr">
@@ -15110,7 +15110,7 @@
       <c r="H110" s="12" t="inlineStr"/>
       <c r="I110" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J110" s="12" t="inlineStr">
@@ -15762,7 +15762,7 @@
       <c r="H125" s="12" t="inlineStr"/>
       <c r="I125" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J125" s="12" t="inlineStr">
@@ -16056,7 +16056,7 @@
       <c r="H132" s="13" t="inlineStr"/>
       <c r="I132" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J132" s="13" t="inlineStr">
@@ -18763,7 +18763,7 @@
       <c r="H195" s="12" t="inlineStr"/>
       <c r="I195" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J195" s="12" t="inlineStr">
@@ -19283,7 +19283,7 @@
       <c r="H207" s="12" t="inlineStr"/>
       <c r="I207" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J207" s="12" t="inlineStr">
@@ -19807,7 +19807,7 @@
       <c r="H220" s="13" t="inlineStr"/>
       <c r="I220" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J220" s="13" t="inlineStr">
@@ -20625,7 +20625,7 @@
       <c r="H239" s="13" t="inlineStr"/>
       <c r="I239" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008116</t>
         </is>
       </c>
       <c r="J239" s="13" t="inlineStr">
@@ -22346,7 +22346,7 @@
       <c r="H9" s="12" t="inlineStr"/>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>VOC4CAT:0007809</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
@@ -22623,7 +22623,7 @@
       <c r="H16" s="13" t="inlineStr"/>
       <c r="I16" s="13" t="inlineStr">
         <is>
-          <t>qudt:Quantity</t>
+          <t>VOC4CAT:0008120</t>
         </is>
       </c>
       <c r="J16" s="13" t="inlineStr">

</xml_diff>